<commit_message>
Automatiza 2 arquivo(s) de processos no painel
</commit_message>
<xml_diff>
--- a/planilhas/LISTA DE PROCESSO PG GREEN.xlsx
+++ b/planilhas/LISTA DE PROCESSO PG GREEN.xlsx
@@ -52,10 +52,10 @@
   <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -333,7 +333,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J52"/>
+  <dimension ref="A1:G56"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -411,7 +411,7 @@
       <c r="F2" t="n">
         <v>39</v>
       </c>
-      <c r="G2" s="3" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>001178</t>
         </is>
@@ -445,7 +445,7 @@
       <c r="F3" t="n">
         <v>7</v>
       </c>
-      <c r="G3" s="3" t="inlineStr">
+      <c r="G3" s="2" t="inlineStr">
         <is>
           <t>001179</t>
         </is>
@@ -479,7 +479,7 @@
       <c r="F4" t="n">
         <v>5</v>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>001180</t>
         </is>
@@ -513,7 +513,7 @@
       <c r="F5" t="n">
         <v>9</v>
       </c>
-      <c r="G5" s="3" t="inlineStr">
+      <c r="G5" s="2" t="inlineStr">
         <is>
           <t>001181</t>
         </is>
@@ -547,7 +547,7 @@
       <c r="F6" t="n">
         <v>3</v>
       </c>
-      <c r="G6" s="3" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>001182</t>
         </is>
@@ -581,7 +581,7 @@
       <c r="F7" t="n">
         <v>1</v>
       </c>
-      <c r="G7" s="3" t="inlineStr">
+      <c r="G7" s="2" t="inlineStr">
         <is>
           <t>001183</t>
         </is>
@@ -615,7 +615,7 @@
       <c r="F8" t="n">
         <v>1</v>
       </c>
-      <c r="G8" s="3" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>001184</t>
         </is>
@@ -649,7 +649,7 @@
       <c r="F9" t="n">
         <v>2</v>
       </c>
-      <c r="G9" s="3" t="inlineStr">
+      <c r="G9" s="2" t="inlineStr">
         <is>
           <t>001185</t>
         </is>
@@ -683,7 +683,7 @@
       <c r="F10" t="n">
         <v>7</v>
       </c>
-      <c r="G10" s="3" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>001186</t>
         </is>
@@ -717,7 +717,7 @@
       <c r="F11" t="n">
         <v>7</v>
       </c>
-      <c r="G11" s="3" t="inlineStr">
+      <c r="G11" s="2" t="inlineStr">
         <is>
           <t>001187</t>
         </is>
@@ -751,7 +751,7 @@
       <c r="F12" t="n">
         <v>30</v>
       </c>
-      <c r="G12" s="3" t="inlineStr">
+      <c r="G12" s="2" t="inlineStr">
         <is>
           <t>001188</t>
         </is>
@@ -785,7 +785,7 @@
       <c r="F13" t="n">
         <v>7</v>
       </c>
-      <c r="G13" s="3" t="inlineStr">
+      <c r="G13" s="2" t="inlineStr">
         <is>
           <t>001189</t>
         </is>
@@ -819,7 +819,7 @@
       <c r="F14" t="n">
         <v>1</v>
       </c>
-      <c r="G14" s="3" t="inlineStr">
+      <c r="G14" s="2" t="inlineStr">
         <is>
           <t>001190</t>
         </is>
@@ -853,7 +853,7 @@
       <c r="F15" t="n">
         <v>2</v>
       </c>
-      <c r="G15" s="3" t="inlineStr">
+      <c r="G15" s="2" t="inlineStr">
         <is>
           <t>001191</t>
         </is>
@@ -887,7 +887,7 @@
       <c r="F16" t="n">
         <v>3</v>
       </c>
-      <c r="G16" s="3" t="inlineStr">
+      <c r="G16" s="2" t="inlineStr">
         <is>
           <t>001192</t>
         </is>
@@ -921,7 +921,7 @@
       <c r="F17" t="n">
         <v>5</v>
       </c>
-      <c r="G17" s="3" t="inlineStr">
+      <c r="G17" s="2" t="inlineStr">
         <is>
           <t>001193</t>
         </is>
@@ -955,7 +955,7 @@
       <c r="F18" t="n">
         <v>17</v>
       </c>
-      <c r="G18" s="3" t="inlineStr">
+      <c r="G18" s="2" t="inlineStr">
         <is>
           <t>001194</t>
         </is>
@@ -989,7 +989,7 @@
       <c r="F19" t="n">
         <v>20</v>
       </c>
-      <c r="G19" s="3" t="inlineStr">
+      <c r="G19" s="2" t="inlineStr">
         <is>
           <t>001195</t>
         </is>
@@ -1023,7 +1023,7 @@
       <c r="F20" t="n">
         <v>1</v>
       </c>
-      <c r="G20" s="3" t="inlineStr">
+      <c r="G20" s="2" t="inlineStr">
         <is>
           <t>001196</t>
         </is>
@@ -1057,7 +1057,7 @@
       <c r="F21" t="n">
         <v>9</v>
       </c>
-      <c r="G21" s="3" t="inlineStr">
+      <c r="G21" s="2" t="inlineStr">
         <is>
           <t>001197</t>
         </is>
@@ -1091,7 +1091,7 @@
       <c r="F22" t="n">
         <v>8</v>
       </c>
-      <c r="G22" s="3" t="inlineStr">
+      <c r="G22" s="2" t="inlineStr">
         <is>
           <t>001198</t>
         </is>
@@ -1125,7 +1125,7 @@
       <c r="F23" t="n">
         <v>14</v>
       </c>
-      <c r="G23" s="3" t="inlineStr">
+      <c r="G23" s="2" t="inlineStr">
         <is>
           <t>001199</t>
         </is>
@@ -1159,7 +1159,7 @@
       <c r="F24" t="n">
         <v>4</v>
       </c>
-      <c r="G24" s="3" t="inlineStr">
+      <c r="G24" s="2" t="inlineStr">
         <is>
           <t>001200</t>
         </is>
@@ -1193,7 +1193,7 @@
       <c r="F25" t="n">
         <v>19</v>
       </c>
-      <c r="G25" s="3" t="inlineStr">
+      <c r="G25" s="2" t="inlineStr">
         <is>
           <t>001201</t>
         </is>
@@ -1227,7 +1227,7 @@
       <c r="F26" t="n">
         <v>13</v>
       </c>
-      <c r="G26" s="3" t="inlineStr">
+      <c r="G26" s="2" t="inlineStr">
         <is>
           <t>001202</t>
         </is>
@@ -1261,7 +1261,7 @@
       <c r="F27" t="n">
         <v>8</v>
       </c>
-      <c r="G27" s="3" t="inlineStr">
+      <c r="G27" s="2" t="inlineStr">
         <is>
           <t>001203</t>
         </is>
@@ -1295,7 +1295,7 @@
       <c r="F28" t="n">
         <v>1</v>
       </c>
-      <c r="G28" s="3" t="inlineStr">
+      <c r="G28" s="2" t="inlineStr">
         <is>
           <t>001204</t>
         </is>
@@ -1329,7 +1329,7 @@
       <c r="F29" t="n">
         <v>1</v>
       </c>
-      <c r="G29" s="3" t="inlineStr">
+      <c r="G29" s="2" t="inlineStr">
         <is>
           <t>001205</t>
         </is>
@@ -1363,7 +1363,7 @@
       <c r="F30" t="n">
         <v>1</v>
       </c>
-      <c r="G30" s="3" t="inlineStr">
+      <c r="G30" s="2" t="inlineStr">
         <is>
           <t>001206</t>
         </is>
@@ -1397,7 +1397,7 @@
       <c r="F31" t="n">
         <v>1</v>
       </c>
-      <c r="G31" s="3" t="inlineStr">
+      <c r="G31" s="2" t="inlineStr">
         <is>
           <t>001207</t>
         </is>
@@ -1431,7 +1431,7 @@
       <c r="F32" t="n">
         <v>1</v>
       </c>
-      <c r="G32" s="3" t="inlineStr">
+      <c r="G32" s="2" t="inlineStr">
         <is>
           <t>001208</t>
         </is>
@@ -1464,7 +1464,7 @@
       <c r="F33" t="n">
         <v>760</v>
       </c>
-      <c r="G33" s="3" t="inlineStr">
+      <c r="G33" s="2" t="inlineStr">
         <is>
           <t>001209</t>
         </is>
@@ -1497,7 +1497,7 @@
       <c r="F34" t="n">
         <v>1760</v>
       </c>
-      <c r="G34" s="3" t="inlineStr">
+      <c r="G34" s="2" t="inlineStr">
         <is>
           <t>001210</t>
         </is>
@@ -1530,7 +1530,7 @@
       <c r="F35" t="n">
         <v>40</v>
       </c>
-      <c r="G35" s="3" t="inlineStr">
+      <c r="G35" s="2" t="inlineStr">
         <is>
           <t>001211</t>
         </is>
@@ -1563,7 +1563,7 @@
       <c r="F36" t="n">
         <v>80</v>
       </c>
-      <c r="G36" s="3" t="inlineStr">
+      <c r="G36" s="2" t="inlineStr">
         <is>
           <t>001212</t>
         </is>
@@ -1596,7 +1596,7 @@
       <c r="F37" t="n">
         <v>40</v>
       </c>
-      <c r="G37" s="3" t="inlineStr">
+      <c r="G37" s="2" t="inlineStr">
         <is>
           <t>001213</t>
         </is>
@@ -1629,7 +1629,7 @@
       <c r="F38" t="n">
         <v>80</v>
       </c>
-      <c r="G38" s="3" t="inlineStr">
+      <c r="G38" s="2" t="inlineStr">
         <is>
           <t>001214</t>
         </is>
@@ -1662,7 +1662,7 @@
       <c r="F39" t="n">
         <v>40</v>
       </c>
-      <c r="G39" s="3" t="inlineStr">
+      <c r="G39" s="2" t="inlineStr">
         <is>
           <t>001215</t>
         </is>
@@ -1695,7 +1695,7 @@
       <c r="F40" t="n">
         <v>40</v>
       </c>
-      <c r="G40" s="3" t="inlineStr">
+      <c r="G40" s="2" t="inlineStr">
         <is>
           <t>001216</t>
         </is>
@@ -1719,7 +1719,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Bandeja</t>
+          <t>Bandeja Amassamento</t>
         </is>
       </c>
       <c r="E41" t="n">
@@ -1728,9 +1728,9 @@
       <c r="F41" t="n">
         <v>40</v>
       </c>
-      <c r="G41" s="3" t="inlineStr">
-        <is>
-          <t>001217</t>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>001253</t>
         </is>
       </c>
     </row>
@@ -1752,18 +1752,18 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Canaleta L 1280</t>
+          <t>Bandeja</t>
         </is>
       </c>
       <c r="E42" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F42" t="n">
-        <v>80</v>
-      </c>
-      <c r="G42" s="3" t="inlineStr">
-        <is>
-          <t>001218</t>
+        <v>40</v>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>001217</t>
         </is>
       </c>
     </row>
@@ -1785,7 +1785,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Canaleta L 180</t>
+          <t>Canaleta L 1280</t>
         </is>
       </c>
       <c r="E43" t="n">
@@ -1794,9 +1794,9 @@
       <c r="F43" t="n">
         <v>80</v>
       </c>
-      <c r="G43" s="3" t="inlineStr">
-        <is>
-          <t>001219</t>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>001218</t>
         </is>
       </c>
     </row>
@@ -1818,18 +1818,18 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Canaleta L 400</t>
+          <t>Canaleta L 180</t>
         </is>
       </c>
       <c r="E44" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F44" t="n">
-        <v>160</v>
-      </c>
-      <c r="G44" s="3" t="inlineStr">
-        <is>
-          <t>001220</t>
+        <v>80</v>
+      </c>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>001219</t>
         </is>
       </c>
     </row>
@@ -1851,18 +1851,18 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Canaleta L 830</t>
+          <t>Canaleta L 400</t>
         </is>
       </c>
       <c r="E45" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F45" t="n">
-        <v>80</v>
-      </c>
-      <c r="G45" s="3" t="inlineStr">
-        <is>
-          <t>001221</t>
+        <v>160</v>
+      </c>
+      <c r="G45" s="2" t="inlineStr">
+        <is>
+          <t>001220</t>
         </is>
       </c>
     </row>
@@ -1884,18 +1884,18 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Chapa 2,65 Parachoque</t>
+          <t>Canaleta L 830</t>
         </is>
       </c>
       <c r="E46" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F46" t="n">
-        <v>160</v>
-      </c>
-      <c r="G46" s="3" t="inlineStr">
-        <is>
-          <t>001222</t>
+        <v>80</v>
+      </c>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>001221</t>
         </is>
       </c>
     </row>
@@ -1917,18 +1917,18 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Gancho Chapa U</t>
+          <t>Chapa 2,65 Parachoque</t>
         </is>
       </c>
       <c r="E47" t="n">
-        <v>63</v>
+        <v>4</v>
       </c>
       <c r="F47" t="n">
-        <v>2520</v>
-      </c>
-      <c r="G47" s="3" t="inlineStr">
-        <is>
-          <t>001223</t>
+        <v>160</v>
+      </c>
+      <c r="G47" s="2" t="inlineStr">
+        <is>
+          <t>001222</t>
         </is>
       </c>
     </row>
@@ -1945,23 +1945,23 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Solda Mig</t>
+          <t>Dobradeira de Chapas</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Corpo</t>
+          <t>Gancho Chapa U</t>
         </is>
       </c>
       <c r="E48" t="n">
-        <v>1</v>
+        <v>63</v>
       </c>
       <c r="F48" t="n">
-        <v>40</v>
-      </c>
-      <c r="G48" s="3" t="inlineStr">
-        <is>
-          <t>001224</t>
+        <v>2520</v>
+      </c>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>001223</t>
         </is>
       </c>
     </row>
@@ -1983,7 +1983,7 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Chaparia Base + Bdj</t>
+          <t>Corpo</t>
         </is>
       </c>
       <c r="E49" t="n">
@@ -1992,9 +1992,9 @@
       <c r="F49" t="n">
         <v>40</v>
       </c>
-      <c r="G49" s="3" t="inlineStr">
-        <is>
-          <t>001225</t>
+      <c r="G49" s="2" t="inlineStr">
+        <is>
+          <t>001224</t>
         </is>
       </c>
     </row>
@@ -2016,7 +2016,7 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Quadro 15X15 Gancho - Frontal e Lateral</t>
+          <t>Chaparia Base + Bdj</t>
         </is>
       </c>
       <c r="E50" t="n">
@@ -2025,9 +2025,9 @@
       <c r="F50" t="n">
         <v>40</v>
       </c>
-      <c r="G50" s="3" t="inlineStr">
-        <is>
-          <t>001226</t>
+      <c r="G50" s="2" t="inlineStr">
+        <is>
+          <t>001225</t>
         </is>
       </c>
     </row>
@@ -2049,7 +2049,7 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Parachoque</t>
+          <t>Quadro 15X15 Gancho - Frontal e Lateral</t>
         </is>
       </c>
       <c r="E51" t="n">
@@ -2058,9 +2058,9 @@
       <c r="F51" t="n">
         <v>40</v>
       </c>
-      <c r="G51" s="3" t="inlineStr">
-        <is>
-          <t>001227</t>
+      <c r="G51" s="2" t="inlineStr">
+        <is>
+          <t>001226</t>
         </is>
       </c>
     </row>
@@ -2082,18 +2082,150 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Gancho + Chapa U</t>
+          <t>Parachoque</t>
         </is>
       </c>
       <c r="E52" t="n">
-        <v>63</v>
+        <v>1</v>
       </c>
       <c r="F52" t="n">
-        <v>2520</v>
-      </c>
-      <c r="G52" s="3" t="inlineStr">
-        <is>
-          <t>001228</t>
+        <v>40</v>
+      </c>
+      <c r="G52" s="2" t="inlineStr">
+        <is>
+          <t>001227</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>GREEN IMPORTADORA</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>PG GREEN</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>Solda Mig</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>Gancho Menor + Chapa U</t>
+        </is>
+      </c>
+      <c r="E53" t="n">
+        <v>19</v>
+      </c>
+      <c r="F53" t="n">
+        <v>760</v>
+      </c>
+      <c r="G53" s="2" t="inlineStr">
+        <is>
+          <t>001254</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>GREEN IMPORTADORA</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>PG GREEN</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Solda Mig</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>Gancho Maior + Chapa U</t>
+        </is>
+      </c>
+      <c r="E54" t="n">
+        <v>44</v>
+      </c>
+      <c r="F54" t="n">
+        <v>1760</v>
+      </c>
+      <c r="G54" s="3" t="inlineStr">
+        <is>
+          <t>001255</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>GREEN IMPORTADORA</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>PG GREEN</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Solda Mig</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Gancho Menor + Trecho Reto</t>
+        </is>
+      </c>
+      <c r="E55" t="n">
+        <v>19</v>
+      </c>
+      <c r="F55" t="n">
+        <v>760</v>
+      </c>
+      <c r="G55" s="3" t="inlineStr">
+        <is>
+          <t>001256</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>GREEN IMPORTADORA</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>PG GREEN</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Solda Mig</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>Gancho Maior + Trecho Reto</t>
+        </is>
+      </c>
+      <c r="E56" t="n">
+        <v>44</v>
+      </c>
+      <c r="F56" t="n">
+        <v>1760</v>
+      </c>
+      <c r="G56" s="3" t="inlineStr">
+        <is>
+          <t>001257</t>
         </is>
       </c>
     </row>

</xml_diff>